<commit_message>
docs+backlog: SIM-536's code fix landed; narrow the ticket to the live re-check
CHANGES.md entry for the fix that shipped in 0fb02ac. BACKLOG.xlsx's SIM-536
row rewritten to reflect that only the re-check of the 2,378 already-loaded
2024 games remains -- the owner is running that personally once fewer other
processes are competing for the database and the live odds API.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -570,10 +570,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-542  (SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet.)</t>
+          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-542  (SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally.)</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="175" customHeight="1">
+    <row r="5" ht="190" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>P1</t>
@@ -622,22 +622,22 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Fix odds being matched to the wrong game</t>
+          <t>Re-check and re-load the already-loaded odds that may have matched the wrong game</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>The system that loads real historical betting odds sometimes attaches the wrong game's odds to a game. It figures out which game a set of odds belongs to using a timestamp recorded in a global time zone, but it should use the official date of the game where it was played. For games that start late at night in Central, Mountain, or Pacific time, this can shift the recorded date to the next day, so the loader pairs that game with a different game between the same two teams the following day. A check found this may affect roughly a quarter to nearly half of games outside the Eastern time zone.</t>
+          <t>The bug that matched betting odds to the wrong game is fixed and merged: the odds loader now uses the game's official local date instead of a global-time-zone timestamp, and a second related bug (always guessing 'game 1' when a doubleheader matched two games) is fixed alongside it. What is left is checking the 2,378 games already loaded for the 2024 season: up to 1,169 of them (any game whose home team is outside the Eastern time zone) could have been affected, though only the ones with a late-evening start actually would have been. Those need to be re-fetched from the real odds provider and reloaded.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>The odds loader matches every game using its official local date, not a global-time-zone timestamp. Doubleheaders are told apart by their scheduled start time. A loaded odds record is rejected if its recorded time is more than about two hours from the game's actual first pitch. The already-loaded 2024 season odds are re-checked and any mismatched games are re-loaded.</t>
+          <t>Every one of the 2,378 already-loaded 2024 games has been checked against the fixed matching logic, and any game whose stored odds came from the wrong game has been reloaded with the correct odds.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Change the matching field from the global-time timestamp to the game's official local date in the odds-loading code (and the same bug in the bullpen-availability loader, which has an identical mistake). Add the first-pitch-time sanity check. Re-run the historical backfill and check the results against what is currently loaded.</t>
+          <t>Run the existing historical-odds loader again for the 2024 season with the fix in place; the loader's own de-duplication already makes a re-run safe to repeat without creating duplicate rows. The owner is running this personally once fewer other processes are competing for the database and the live odds API — this should not be started by anyone else in the meantime.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sim-537): record the pitcher and manager point-in-time landing
Updates CHANGES.md and BACKLOG.xlsx to reflect that SIM-537's pitcher
and manager groupings are done (commit 8aa13ae). The ticket stays
open: baserunner, catcher, and fielder are unchanged and still need
their own point-in-time work, scoped in
docs/audit/2026-09-10-savant-point-in-time-data.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -573,7 +573,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-542  (SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally.)</t>
+          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-542  (SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally. SIM-537's pitcher and manager groups landed 2026-09-11; baserunner, catcher, and fielder stay open.)</t>
         </is>
       </c>
     </row>
@@ -654,22 +654,22 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Extend point-in-time cutoffs to the remaining player profiles</t>
+          <t>Extend point-in-time cutoffs to the remaining player profiles (pitcher and manager DONE)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Two recent changes made sure the simulator, when replaying a game from the past, cannot use information recorded after that game — first for a batter's own statistics, then for the pool of real plays the simulator draws from. Several other player-measurement types were not part of either fix: a fielder's or catcher's throwing strength, sprint speed, pop time, and most base-running measurements are still calculated from an entire season at once, with no way to cut them off at a specific date. That means a simulation of an early-season game can still be quietly informed by that same player's performance from later in the season.</t>
+          <t>Two recent changes made sure the simulator, when replaying a game from the past, cannot use information recorded after that game — first for a batter's own statistics, then for the pool of real plays the simulator draws from. Five more player-measurement groups were not part of either fix: pitcher, manager, fielder, catcher, and baserunner. The pitcher and manager groups are now done: both read only our own data (no outside data source), so a plain date cutoff was enough. The other three groups still calculate some measurements from an entire season at once, with no way to cut them off at a specific date. That means a simulation of an early-season game can still be quietly informed by that same player's performance from later in the season.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Every player-measurement input the simulator reads for pitchers, fielders, catchers, and baserunners can be built as of a specific date, using the same rule already applied to batters: a season that ended before the cutoff counts in full, and only the season containing the cutoff is trimmed to what happened through that date. The system refuses to run with a mismatched cutoff across different measurement types.</t>
+          <t>Every player-measurement input the simulator reads for fielders, catchers, and baserunners can be built as of a specific date, using the same rule already applied to batters, pitchers, and managers: a season that ended before the cutoff counts in full, and only the season containing the cutoff is trimmed to what happened through that date. The system refuses to run with a mismatched cutoff across different measurement types. (Pitcher and manager already meet this bar and are verified by 24 automated tests.)</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Apply the same pattern already built for batters — a per-source "as of" date column, a cutoff rule on top of it, and a check after building that confirms nothing dated after the cutoff was used — to the remaining profile builders (fielder, catcher, baserunner, pitcher, manager).</t>
+          <t>DONE for pitcher and manager: a per-source "as of" date column, a cutoff rule on top of it, and a check after building that confirms nothing dated after the cutoff was used. Still to do, one group at a time: baserunner and catcher mix our own data with season-only outside measurements (sprint speed, throwing strength) that need a fallback to the most recent full season when a mid-season cutoff is requested; fielder needs the same treatment applied separately across its seven measurement types, since they draw from different sources. All three are scoped in docs/audit/2026-09-10-savant-point-in-time-data.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sim-529,530): close both tickets on the board
Removed from the open list (28 -> 26) and named in the subtitle beside the
other 2026-09-10 closures. The next free id is asserted before and after the
rewrite and passes through untouched at SIM-542 — the SIM-528 closure clobbered
it and this script now refuses to run if the number is not what it expects.

The changelog entry landed earlier in 3a9b6b1; this is the board half.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -107,8 +112,28 @@
         <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E26B0A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF9000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,11 +155,12 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,6 +198,34 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -570,8 +624,8 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-542  (SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally. SIM-537's pitcher and manager groups landed 2026-09-11; baserunner, catcher, and fielder stay open.)</t>
         </is>
@@ -610,927 +664,872 @@
       </c>
     </row>
     <row r="5" ht="190" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>SIM-536</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Re-check and re-load the already-loaded odds that may have matched the wrong game</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>The bug that matched betting odds to the wrong game is fixed and merged: the odds loader now uses the game's official local date instead of a global-time-zone timestamp, and a second related bug (always guessing 'game 1' when a doubleheader matched two games) is fixed alongside it. What is left is checking the 2,378 games already loaded for the 2024 season: up to 1,169 of them (any game whose home team is outside the Eastern time zone) could have been affected, though only the ones with a late-evening start actually would have been. Those need to be re-fetched from the real odds provider and reloaded.</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>Every one of the 2,378 already-loaded 2024 games has been checked against the fixed matching logic, and any game whose stored odds came from the wrong game has been reloaded with the correct odds.</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>Run the existing historical-odds loader again for the 2024 season with the fix in place; the loader's own de-duplication already makes a re-run safe to repeat without creating duplicate rows. The owner is running this personally once fewer other processes are competing for the database and the live odds API — this should not be started by anyone else in the meantime.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="190" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>SIM-537</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Extend point-in-time cutoffs to the remaining player profiles (pitcher and manager DONE)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>Two recent changes made sure the simulator, when replaying a game from the past, cannot use information recorded after that game — first for a batter's own statistics, then for the pool of real plays the simulator draws from. Five more player-measurement groups were not part of either fix: pitcher, manager, fielder, catcher, and baserunner. The pitcher and manager groups are now done: both read only our own data (no outside data source), so a plain date cutoff was enough. The other three groups still calculate some measurements from an entire season at once, with no way to cut them off at a specific date. That means a simulation of an early-season game can still be quietly informed by that same player's performance from later in the season.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>Every player-measurement input the simulator reads for fielders, catchers, and baserunners can be built as of a specific date, using the same rule already applied to batters, pitchers, and managers: a season that ended before the cutoff counts in full, and only the season containing the cutoff is trimmed to what happened through that date. The system refuses to run with a mismatched cutoff across different measurement types. (Pitcher and manager already meet this bar and are verified by 24 automated tests.)</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>DONE for pitcher and manager: a per-source "as of" date column, a cutoff rule on top of it, and a check after building that confirms nothing dated after the cutoff was used. Still to do, one group at a time: baserunner and catcher mix our own data with season-only outside measurements (sprint speed, throwing strength) that need a fallback to the most recent full season when a mid-season cutoff is requested; fielder needs the same treatment applied separately across its seven measurement types, since they draw from different sources. All three are scoped in docs/audit/2026-09-10-savant-point-in-time-data.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="175" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>SIM-538</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Build the sim-vs-closing-line accuracy comparison</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>Build the platform's new way of checking whether its predictions are good: for every game or player prop where a final ("closing") betting price is available, compare the simulator's own predicted probability and the market's probability (with the bookmaker's built-in margin removed) against what actually happened, and see which one was more accurate. This replaces trying to catch a betting line's price movement, which does not work well for this platform because the simulator cannot make a prediction until both teams' starting lineups are announced — which is after betting lines first open.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>For a slate of completed games with closing odds, the tool reports, per market and player-prop type: how many games/props were compared, how much more (or less) accurate the simulator was than the market on average, and whether that difference is likely real or could be chance.</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>Reuse the existing game-replay and odds-reading code, the existing bookmaker-margin-removal math, and the existing accuracy-scoring math already built elsewhere in the platform. The only new code is the piece that runs both the simulator's number and the market's number through the same accuracy score and reports the difference. Keep the platform's old betting-line-movement report available as a secondary, clearly-labeled reference rather than deleting it.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="160" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>SIM-539</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Add real statistical confidence to the accuracy comparison</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>Right now, when the platform reports a betting-accuracy result, it reports a single number with no sense of whether that number is reliable or just noise. A result from a small number of games can look like real skill purely by chance.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>Every reported accuracy comparison comes with a range showing how confident the platform is in that number, and the platform states, per market, the smallest number of games needed before a result should be trusted at all.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>Because the simulator's score and the market's score come from the exact same games, use a statistical method built for comparing paired results (for example, a paired bootstrap or a paired significance test on the per-game score difference) rather than treating the two as unrelated samples — this needs fewer games to detect a real difference. Set and document a minimum sample size per market before publishing a headline number for it.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="115" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>SIM-540</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Report the hypothetical dollar return alongside the accuracy score</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>An accuracy score is useful for the team but harder for a non-technical reader to judge. Add a companion report: whenever the simulator's probability disagrees with the market's probability by more than a set amount, calculate what the return would have been on a bet placed at the closing price, and add up that hypothetical return across many games.</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>The accuracy-comparison tool can optionally output an estimated return on investment, with a confidence range, for a chosen disagreement threshold.</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>Reuse the platform's existing bet-value calculation; aggregate it only over the bets that clear the disagreement threshold, using the same real-outcome data the accuracy comparison already reads.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="130" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>SIM-541</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Find and use all the closing-line odds data already being collected</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>The current historical odds data only covers games where both an opening and a closing price were captured and matched. The platform's odds-collection process is believed to capture closing prices on many more games than that, without always having a matching opening price. Since the new accuracy comparison only needs the closing price, this may unlock a much bigger set of games to test against — nobody has checked.</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>A clear count of how many additional games/props have a usable closing price today that the current backtest does not use, and the accuracy-comparison tool updated to use all of them, not only the subset that also has a matched opening price.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>Audit the current odds-scraping and storage path end to end to see what is actually captured versus what the backtest currently reads. Relax the backtest's game-selection to require only a closing price, not both.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="250" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>SIM-421</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Add the prop-bet types the market already offers but the platform does not price</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>A live check of the platform's own odds source (2026-09-11, two days of real games) found six batter prop types posted on nearly every game that the platform does not price at all: singles, doubles, triples, runs scored, stolen bases, and a combined runs+hits+RBIs bet. Together they had more real, gradable bets than all seven of the platform's current prop types combined, over the same two days. A pitcher prop (outs recorded) and a likely-mislabeled one (hits allowed, separate from batter hits) were also found unpriced.</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>The platform produces its own price projection for singles, doubles, triples, runs, steals, runs+hits+RBIs, and pitcher outs recorded, matched to real posted odds for each. Lower-volume game-segment markets (first/fifth-inning splits, team totals) are scoped as a follow-on, not required for this ticket.</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Almost none of this needs new simulation logic: the simulator's own per-player game record already tracks doubles, triples, runs, and stolen bases on every simulated game, and a pitcher's outs-recorded projection is already built and just not connected to real odds. The work is adding a probability-distribution wrapper for each new stat (matching the pattern the existing seven props already use), adding each to the odds-loading vocabulary, and confirming the odds loader does not confuse pitcher 'hits allowed' with batter 'hits', since the market data carries them as two separate markets. See docs/audit/2026-09-11-sim421-prop-market-scrape.md for the full breakdown and the recommended build order.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="160" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="12" ht="130" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>SIM-529</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Add physical swing and stance measurements to batter matching</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>The simulator decides how similar two batters are using only the results they produced: how often they miss, walk, or pull the ball. Baseball Savant now publishes how each batter actually swings, including bat speed, swing length, the angle of the swing, and how the batter stands in the batter's box. Testing on our own data shows several of these repeat from season to season more reliably than any measurement the platform uses today, and that three of them describe something our current measurements cannot detect at all.</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Ten new physical measurements are stored for every batter season, the batter-matching model uses them with tuned weights, and the platform's standard accuracy checks still pass.</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Load the three Savant swing files, add the columns to the batter profile, add a new group of physical measurements to the matching model, tune its weight and re-run the standard accuracy check. Needs the Savant loader first. The evidence and the exact ten columns are in docs/audit/2026-09-10-savant-leaderboard-data-audit.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="130" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>SIM-518</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Fit and turn on new pitch-realism factors</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>The team built three new pieces of information the simulator could use when picking each pitch: how tired the pitcher is, which side of the plate the batter stands on, and how similar a batted ball is to the pitch that produced it. All three are built and the supporting data has been rebuilt, but none are turned on because their strength has not been tuned against real outcomes and they have not been tested together.</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Each of the three factors has a tuned strength setting, and a test run on the platform's standard 45-game set passes with all three turned on.</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Tune each factor's strength against the platform's historical data, then run the standard 45-game test with all three enabled and fix anything that fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="160" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>SIM-530</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Fill three empty player-measurement blocks</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Three sets of player measurements that the matching models actively weight contain no data at all. The worst is the outfielder's throwing arm, which counts for 30% of an outfielder's similarity score and is empty for every outfielder in the database. The catcher's arm strength is also empty despite carrying a heavy weight, and the first baseman's scoop rate is missing for most players. Baseball Savant publishes all three.</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>The outfield arm, catcher arm and first-base scoop measurements hold real values for every season the simulator draws from, and the models that weight them produce different scores than they do today.</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Load Savant's arm strength, arm value, catcher pop time, catcher throwing and first-base receiving files, then join them into the fielder and catcher profiles. This absorbs the retired fielder arm-strength ticket (SIM-521), which was removed from the board on 2026-09-10. Needs the Savant loader first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="130" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>SIM-427</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Use each team's real manager tendencies for pitching changes</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>When the simulator decides whether a manager would pull the starting pitcher for a reliever, it currently uses one league-wide average tendency for every team instead of that team's real, historical tendency. The real per-team data already exists elsewhere in the system; it just is not connected to this decision yet. A related gap: some rare manager choices, like calling for a bunt, are shown to users as if they happened even though the simulator does not actually change the play's outcome for them.</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>The pitching-change decision uses each team's own manager tendencies instead of one shared league average, and the resulting pitching-change rate still matches real-world data within the platform's accuracy band.</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Connect the already-computed per-team manager data into the pitching-change decision, and separately decide whether to remove or properly implement the bunt/pitch-out narration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="160" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>SIM-518</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Fit and turn on new pitch-realism factors</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>The team built three new pieces of information the simulator could use when picking each pitch: how tired the pitcher is, which side of the plate the batter stands on, and how similar a batted ball is to the pitch that produced it. All three are built and the supporting data has been rebuilt, but none are turned on because their strength has not been tuned against real outcomes and they have not been tested together.</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Each of the three factors has a tuned strength setting, and a test run on the platform's standard 45-game set passes with all three turned on.</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Tune each factor's strength against the platform's historical data, then run the standard 45-game test with all three enabled and fix anything that fails.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="160" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>SIM-427</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Use each team's real manager tendencies for pitching changes</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>When the simulator decides whether a manager would pull the starting pitcher for a reliever, it currently uses one league-wide average tendency for every team instead of that team's real, historical tendency. The real per-team data already exists elsewhere in the system; it just is not connected to this decision yet. A related gap: some rare manager choices, like calling for a bunt, are shown to users as if they happened even though the simulator does not actually change the play's outcome for them.</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>The pitching-change decision uses each team's own manager tendencies instead of one shared league average, and the resulting pitching-change rate still matches real-world data within the platform's accuracy band.</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Connect the already-computed per-team manager data into the pitching-change decision, and separately decide whether to remove or properly implement the bunt/pitch-out narration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="160" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>SIM-531</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Add lead distance to the stolen-base and baserunning models</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>When the simulator decides whether a runner tries to steal, it leans heavily on how similar the live runner, pitcher and catcher are to the ones in past plays. Those comparisons use only results today: how often the runner went, and how often he was safe. Savant publishes how far each runner actually leads off the base, in feet, and how big a lead each pitcher allows. It also publishes how often a runner tried for an extra base out of the chances he had, which is a denominator the platform does not have.</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>Lead distance and extra-base opportunity rates are stored for runners and pitchers, the stealing and advancement models use them, and the standard accuracy checks still pass.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>Load Savant's basestealing run value, pitcher running game and baserunning files. Add the new measurements to the runner and pitcher profiles, tune their weights and re-run the checks. Needs the Savant loader first.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="100" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="15" ht="100" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>SIM-526</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E15" s="19" t="inlineStr">
         <is>
           <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="100" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="16" ht="100" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>SIM-484</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Model the 'dropped third strike' play</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>Under baseball's real rules, if the catcher fails to cleanly catch a third strike, the batter can sometimes try to run to first base instead of being automatically out. The simulator does not model this rule at all; it always treats a third strike as a simple out. This is a rare but currently missing type of play.</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>The simulator can produce a 'dropped third strike' play in the situations where a real one is possible, at a rate consistent with real baseball data.</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>No detailed implementation plan exists yet; the next step is to design how this fits into the existing pitch and catcher outcome logic.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="115" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="17" ht="115" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>SIM-532</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Add fielder split-by-batter-hand and first-step measurements</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>The simulator compares fielders using range and error rates it computes itself. Savant adds two things the platform cannot compute: how well each fielder performs against left-handed versus right-handed batters, and how much of an outfielder's range comes from his reaction, his acceleration and the route he takes. Both would make the choice of which past play to copy more realistic.</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>The fielder profile carries the batter-hand split and the outfield first-step measurements, and the fielding model uses them without breaking the accuracy checks.</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>Load Savant's outs above average and outfield jump files, add the columns to the fielder profile, tune the weights and re-run the checks. Needs the Savant loader first.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="130" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="18" ht="130" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>SIM-533</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Add pitcher arm angle and spin-shape measurements</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>The simulator groups similar pitchers by the speed and movement of their pitches. Savant publishes the pitcher's arm angle in degrees, and how much of each pitch's spin actually moves the ball. Both describe the pitcher physically rather than by his results. This is the least certain of the Savant additions, because the pitcher model deliberately leaves out where the ball is released, and arm angle is closely related to that.</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>A decision is recorded on whether arm angle belongs in the pitcher model, and any measurements that are adopted are stored, weighted and checked.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>Review the release-point decision first. If arm angle is accepted, load Savant's arm angle, active spin and spin direction files, add them to the pitcher profile, then tune and re-check.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="160" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="19" ht="160" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>SIM-478/479/480</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Certify the outfield-fence / home-run boundary logic</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>When a batted ball heads toward the outfield wall, the simulator checks that specific ballpark's real fence distance and height to decide whether it is a home run or stays in play. The three pieces of this feature (a table of every park's fence measurements, a model of how far a ball actually flies, and the final wall-play check) have been built and wired in as part of a recent redesign, but they are still marked as pending their own dedicated accuracy test before being called fully certified.</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>The fence-boundary logic passes a dedicated accuracy check on the platform's standard test set for home-run and wall-play outcomes.</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>Run the standard accuracy test focused on home-run and wall-play outcomes, and close out any tuning it surfaces.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="145" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="20" ht="145" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>SIM-451</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Re-check that every play-selection group has enough data</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>The simulator picks each pitch by first grouping similar past pitches into small buckets (based on things like the count and which bases have runners), then drawing an outcome from the most similar bucket. This check re-measures how many real pitches fall into each of the roughly 2,880 buckets, to make sure none is so small that its draw becomes unreliable. It needs to be re-run because the number of buckets is about to double once the new pitch-realism factors go live.</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>The bucket-size check has been re-run on the current data, and the platform has a documented minimum acceptable bucket size based on the results.</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>Re-run the existing bucket-coverage measurement script once the pitch-realism-factor rebuild finishes, and use its results to set the minimum bucket size.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="130" customHeight="1">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="21" ht="130" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>SIM-519</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Build the live, schedule-driven game day view</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>The public-facing screen that lists all of today's games should pull its list directly from Major League Baseball's own public schedule and mark each game as upcoming, in progress, or finished. Right now it pulls its game list only from the platform's own database, which can miss games or show stale information. This is a multi-part project; each part can be finished and checked off on its own.</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>The day view lists every game the league's real schedule shows for that day, with the correct status, sourced live from the league rather than only from the platform's own stored data.</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>Build a connection to the league's public schedule feed, use it to drive the list of games shown, and keep layering the platform's simulations, projections, and odds on top of that live list.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="115" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="22" ht="115" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>SIM-524</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Fix the database lock that blocks nightly data rebuilds</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="100" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="23" ht="100" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>SIM-443d</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
+    <row r="24" ht="85" customHeight="1">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>SIM-443e</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Turn on the read-only database connection for the SQL tool</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="85" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>SIM-443a</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Stop exposing database ports to the network</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="85" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>SIM-443e</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="85" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>SIM-443b</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>Remove the default database password and admin access</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="100" customHeight="1">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>SIM-443a</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Stop exposing database ports to the network</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="85" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>SIM-443c</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Require login on the API</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="115" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>SIM-443b</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Remove the default database password and admin access</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>SIM-443f</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>Secure the shared cache (Redis)</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="100" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>SIM-443c</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Require login on the API</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="115" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>SIM-525</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Set up scheduled backups</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="100" customHeight="1">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>SIM-443f</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Secure the shared cache (Redis)</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="100" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>SIM-525</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Set up scheduled backups</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="100" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>SIM-493</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Break up the oversized simulation-loop code file</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (over 3,400 lines) as more features were added over time. This makes it harder to review and maintain safely. The team has deliberately postponed this cleanup until the in-progress pitch-speed and pitch-realism work settles down.</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>The simulation-loop code is split into smaller, clearly-scoped files with no change in what the simulator actually does, confirmed by the platform's existing automated tests.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F30" s="19" t="inlineStr">
         <is>
           <t>Wait until the pitch-bucketing and pitch-realism-factor tickets are settled, then split the file into smaller modules by responsibility.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="22" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="22" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>P0 — drop everything</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C32" s="25" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D32" s="26" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
+      <c r="F32" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs(sim-539): close the ticket in the changelog and backlog
Records SIM-539's closure: the stated minimum sample size and
game-clustered confidence read for both CLV reports, the adversarial
review's critical finding (a tiny lucky sample reading as fully
resolved) and how it was fixed, and the smaller fixes alongside it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG.xlsx
+++ b/BACKLOG.xlsx
@@ -606,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -627,7 +627,7 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-543  (SIM-542 closed 2026-09-11 — the two fielder placeholder tables now name their columns the same way the real builders do. SIM-538 CLOSED 2026-09-11 — the sim-vs-closing-line accuracy comparison is built and shipped, replacing Closing Line Value as the gold-standard metric; an adversarial review found and fixed a real cross-game point-in-time data leak before it landed. SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally. SIM-537 CLOSED 2026-09-11 — every player-measurement group the simulator reads (batter, pitcher, manager, baserunner, catcher, fielder) can now be built as of a specific date.)</t>
+          <t>Updated 2026-09-11. Ranked by priority. The frozen closed-ticket history lives at docs/archive/BACKLOG-history.md.  NEXT FREE TICKET ID: SIM-544  (SIM-538 CLOSED 2026-09-11 — the sim-vs-closing-line accuracy comparison shipped, and SIM-539 CLOSED THE SAME DAY — both reports now state a minimum sample size and a game-clustered confidence read; an adversarial review found and fixed a real "a tiny lucky sample reads as fully resolved" gap before it landed. SIM-542 closed 2026-09-11 — the two fielder placeholder tables now name their columns the same way the real builders do. SIM-538 CLOSED 2026-09-11 — the sim-vs-closing-line accuracy comparison is built and shipped, replacing Closing Line Value as the gold-standard metric; an adversarial review found and fixed a real cross-game point-in-time data leak before it landed. SIM-534/535/528 closed 2026-09-10; SIM-527 and SIM-429 closed 2026-09-10 — the pool-totals shortfall finding behind both is no longer trusted evidence under the new sim-vs-closing-line accuracy metric, so there is nothing confirmed to refit yet. SIM-536's code fix landed 2026-09-11; its remaining scope is a live re-check the owner is running personally. SIM-537 CLOSED 2026-09-11 — every player-measurement group the simulator reads (batter, pitcher, manager, baserunner, catcher, fielder) can now be built as of a specific date.)</t>
         </is>
       </c>
     </row>
@@ -704,27 +704,27 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>SIM-539</t>
+          <t>SIM-540</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Add real statistical confidence to the accuracy comparison</t>
+          <t>Report the hypothetical dollar return alongside the accuracy score</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Right now, when the platform reports a betting-accuracy result, it reports a single number with no sense of whether that number is reliable or just noise. A result from a small number of games can look like real skill purely by chance.</t>
+          <t>An accuracy score is useful for the team but harder for a non-technical reader to judge. Add a companion report: whenever the simulator's probability disagrees with the market's probability by more than a set amount, calculate what the return would have been on a bet placed at the closing price, and add up that hypothetical return across many games.</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Every reported accuracy comparison comes with a range showing how confident the platform is in that number, and the platform states, per market, the smallest number of games needed before a result should be trusted at all.</t>
+          <t>The accuracy-comparison tool can optionally output an estimated return on investment, with a confidence range, for a chosen disagreement threshold.</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>Because the simulator's score and the market's score come from the exact same games, use a statistical method built for comparing paired results (for example, a paired bootstrap or a paired significance test on the per-game score difference) rather than treating the two as unrelated samples — this needs fewer games to detect a real difference. Set and document a minimum sample size per market before publishing a headline number for it.</t>
+          <t>Reuse the platform's existing bet-value calculation; aggregate it only over the bets that clear the disagreement threshold, using the same real-outcome data the accuracy comparison already reads.</t>
         </is>
       </c>
     </row>
@@ -736,27 +736,27 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>SIM-540</t>
+          <t>SIM-541</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Report the hypothetical dollar return alongside the accuracy score</t>
+          <t>Find and use all the closing-line odds data already being collected</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>An accuracy score is useful for the team but harder for a non-technical reader to judge. Add a companion report: whenever the simulator's probability disagrees with the market's probability by more than a set amount, calculate what the return would have been on a bet placed at the closing price, and add up that hypothetical return across many games.</t>
+          <t>The current historical odds data only covers games where both an opening and a closing price were captured and matched. The platform's odds-collection process is believed to capture closing prices on many more games than that, without always having a matching opening price. Since the new accuracy comparison only needs the closing price, this may unlock a much bigger set of games to test against — nobody has checked.</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>The accuracy-comparison tool can optionally output an estimated return on investment, with a confidence range, for a chosen disagreement threshold.</t>
+          <t>A clear count of how many additional games/props have a usable closing price today that the current backtest does not use, and the accuracy-comparison tool updated to use all of them, not only the subset that also has a matched opening price.</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Reuse the platform's existing bet-value calculation; aggregate it only over the bets that clear the disagreement threshold, using the same real-outcome data the accuracy comparison already reads.</t>
+          <t>Audit the current odds-scraping and storage path end to end to see what is actually captured versus what the backtest currently reads. Relax the backtest's game-selection to require only a closing price, not both.</t>
         </is>
       </c>
     </row>
@@ -768,27 +768,27 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>SIM-541</t>
+          <t>SIM-421</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Find and use all the closing-line odds data already being collected</t>
+          <t>Add the prop-bet types the market already offers but the platform does not price</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>The current historical odds data only covers games where both an opening and a closing price were captured and matched. The platform's odds-collection process is believed to capture closing prices on many more games than that, without always having a matching opening price. Since the new accuracy comparison only needs the closing price, this may unlock a much bigger set of games to test against — nobody has checked.</t>
+          <t>A live check of the platform's own odds source (2026-09-11, two days of real games) found six batter prop types posted on nearly every game that the platform does not price at all: singles, doubles, triples, runs scored, stolen bases, and a combined runs+hits+RBIs bet. Together they had more real, gradable bets than all seven of the platform's current prop types combined, over the same two days. A pitcher prop (outs recorded) and a likely-mislabeled one (hits allowed, separate from batter hits) were also found unpriced.</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>A clear count of how many additional games/props have a usable closing price today that the current backtest does not use, and the accuracy-comparison tool updated to use all of them, not only the subset that also has a matched opening price.</t>
+          <t>The platform produces its own price projection for singles, doubles, triples, runs, steals, runs+hits+RBIs, and pitcher outs recorded, matched to real posted odds for each. Lower-volume game-segment markets (first/fifth-inning splits, team totals) are scoped as a follow-on, not required for this ticket.</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>Audit the current odds-scraping and storage path end to end to see what is actually captured versus what the backtest currently reads. Relax the backtest's game-selection to require only a closing price, not both.</t>
+          <t>Almost none of this needs new simulation logic: the simulator's own per-player game record already tracks doubles, triples, runs, and stolen bases on every simulated game, and a pitcher's outs-recorded projection is already built and just not connected to real odds. The work is adding a probability-distribution wrapper for each new stat (matching the pattern the existing seven props already use), adding each to the odds-loading vocabulary, and confirming the odds loader does not confuse pitcher 'hits allowed' with batter 'hits', since the market data carries them as two separate markets. See docs/audit/2026-09-11-sim421-prop-market-scrape.md for the full breakdown and the recommended build order.</t>
         </is>
       </c>
     </row>
@@ -800,27 +800,27 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>SIM-421</t>
+          <t>SIM-518</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Add the prop-bet types the market already offers but the platform does not price</t>
+          <t>Fit and turn on new pitch-realism factors</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>A live check of the platform's own odds source (2026-09-11, two days of real games) found six batter prop types posted on nearly every game that the platform does not price at all: singles, doubles, triples, runs scored, stolen bases, and a combined runs+hits+RBIs bet. Together they had more real, gradable bets than all seven of the platform's current prop types combined, over the same two days. A pitcher prop (outs recorded) and a likely-mislabeled one (hits allowed, separate from batter hits) were also found unpriced.</t>
+          <t>The team built three new pieces of information the simulator could use when picking each pitch: how tired the pitcher is, which side of the plate the batter stands on, and how similar a batted ball is to the pitch that produced it. All three are built and the supporting data has been rebuilt, but none are turned on because their strength has not been tuned against real outcomes and they have not been tested together.</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>The platform produces its own price projection for singles, doubles, triples, runs, steals, runs+hits+RBIs, and pitcher outs recorded, matched to real posted odds for each. Lower-volume game-segment markets (first/fifth-inning splits, team totals) are scoped as a follow-on, not required for this ticket.</t>
+          <t>Each of the three factors has a tuned strength setting, and a test run on the platform's standard 45-game set passes with all three turned on.</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
         <is>
-          <t>Almost none of this needs new simulation logic: the simulator's own per-player game record already tracks doubles, triples, runs, and stolen bases on every simulated game, and a pitcher's outs-recorded projection is already built and just not connected to real odds. The work is adding a probability-distribution wrapper for each new stat (matching the pattern the existing seven props already use), adding each to the odds-loading vocabulary, and confirming the odds loader does not confuse pitcher 'hits allowed' with batter 'hits', since the market data carries them as two separate markets. See docs/audit/2026-09-11-sim421-prop-market-scrape.md for the full breakdown and the recommended build order.</t>
+          <t>Tune each factor's strength against the platform's historical data, then run the standard 45-game test with all three enabled and fix anything that fails.</t>
         </is>
       </c>
     </row>
@@ -832,27 +832,27 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>SIM-518</t>
+          <t>SIM-427</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Fit and turn on new pitch-realism factors</t>
+          <t>Use each team's real manager tendencies for pitching changes</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>The team built three new pieces of information the simulator could use when picking each pitch: how tired the pitcher is, which side of the plate the batter stands on, and how similar a batted ball is to the pitch that produced it. All three are built and the supporting data has been rebuilt, but none are turned on because their strength has not been tuned against real outcomes and they have not been tested together.</t>
+          <t>When the simulator decides whether a manager would pull the starting pitcher for a reliever, it currently uses one league-wide average tendency for every team instead of that team's real, historical tendency. The real per-team data already exists elsewhere in the system; it just is not connected to this decision yet. A related gap: some rare manager choices, like calling for a bunt, are shown to users as if they happened even though the simulator does not actually change the play's outcome for them.</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Each of the three factors has a tuned strength setting, and a test run on the platform's standard 45-game set passes with all three turned on.</t>
+          <t>The pitching-change decision uses each team's own manager tendencies instead of one shared league average, and the resulting pitching-change rate still matches real-world data within the platform's accuracy band.</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>Tune each factor's strength against the platform's historical data, then run the standard 45-game test with all three enabled and fix anything that fails.</t>
+          <t>Connect the already-computed per-team manager data into the pitching-change decision, and separately decide whether to remove or properly implement the bunt/pitch-out narration.</t>
         </is>
       </c>
     </row>
@@ -864,59 +864,59 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>SIM-427</t>
+          <t>SIM-531</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Use each team's real manager tendencies for pitching changes</t>
+          <t>Add lead distance to the stolen-base and baserunning models</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>When the simulator decides whether a manager would pull the starting pitcher for a reliever, it currently uses one league-wide average tendency for every team instead of that team's real, historical tendency. The real per-team data already exists elsewhere in the system; it just is not connected to this decision yet. A related gap: some rare manager choices, like calling for a bunt, are shown to users as if they happened even though the simulator does not actually change the play's outcome for them.</t>
+          <t>When the simulator decides whether a runner tries to steal, it leans heavily on how similar the live runner, pitcher and catcher are to the ones in past plays. Those comparisons use only results today: how often the runner went, and how often he was safe. Savant publishes how far each runner actually leads off the base, in feet, and how big a lead each pitcher allows. It also publishes how often a runner tried for an extra base out of the chances he had, which is a denominator the platform does not have.</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>The pitching-change decision uses each team's own manager tendencies instead of one shared league average, and the resulting pitching-change rate still matches real-world data within the platform's accuracy band.</t>
+          <t>Lead distance and extra-base opportunity rates are stored for runners and pitchers, the stealing and advancement models use them, and the standard accuracy checks still pass.</t>
         </is>
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>Connect the already-computed per-team manager data into the pitching-change decision, and separately decide whether to remove or properly implement the bunt/pitch-out narration.</t>
+          <t>Load Savant's basestealing run value, pitcher running game and baserunning files. Add the new measurements to the runner and pitcher profiles, tune their weights and re-run the checks. Needs the Savant loader first.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="130" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>SIM-531</t>
+          <t>SIM-526</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>Add lead distance to the stolen-base and baserunning models</t>
+          <t>Turn on the catcher pitch-receiving factor</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>When the simulator decides whether a runner tries to steal, it leans heavily on how similar the live runner, pitcher and catcher are to the ones in past plays. Those comparisons use only results today: how often the runner went, and how often he was safe. Savant publishes how far each runner actually leads off the base, in feet, and how big a lead each pitcher allows. It also publishes how often a runner tried for an extra base out of the chances he had, which is a denominator the platform does not have.</t>
+          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Lead distance and extra-base opportunity rates are stored for runners and pitchers, the stealing and advancement models use them, and the standard accuracy checks still pass.</t>
+          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
         </is>
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Load Savant's basestealing run value, pitcher running game and baserunning files. Add the new measurements to the runner and pitcher profiles, tune their weights and re-run the checks. Needs the Savant loader first.</t>
+          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
         </is>
       </c>
     </row>
@@ -928,27 +928,27 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>SIM-526</t>
+          <t>SIM-484</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Turn on the catcher pitch-receiving factor</t>
+          <t>Model the 'dropped third strike' play</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>The team built a feature that scores how good each catcher is at making a borderline pitch look like a strike (sometimes called 'framing'), which can affect whether a close pitch is called a ball or a strike. It is built and tested but currently switched off in the live simulator, pending a decision on how strongly to weight it.</t>
+          <t>Under baseball's real rules, if the catcher fails to cleanly catch a third strike, the batter can sometimes try to run to first base instead of being automatically out. The simulator does not model this rule at all; it always treats a third strike as a simple out. This is a rare but currently missing type of play.</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>The catcher pitch-receiving factor has a chosen strength setting and is switched on in production without breaking any of the platform's existing accuracy checks.</t>
+          <t>The simulator can produce a 'dropped third strike' play in the situations where a real one is possible, at a rate consistent with real baseball data.</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Decide the weight to give this factor based on testing already done, turn it on, and confirm the standard accuracy checks still pass.</t>
+          <t>No detailed implementation plan exists yet; the next step is to design how this fits into the existing pitch and catcher outcome logic.</t>
         </is>
       </c>
     </row>
@@ -960,27 +960,27 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>SIM-484</t>
+          <t>SIM-532</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Model the 'dropped third strike' play</t>
+          <t>Add fielder split-by-batter-hand and first-step measurements</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Under baseball's real rules, if the catcher fails to cleanly catch a third strike, the batter can sometimes try to run to first base instead of being automatically out. The simulator does not model this rule at all; it always treats a third strike as a simple out. This is a rare but currently missing type of play.</t>
+          <t>The simulator compares fielders using range and error rates it computes itself. Savant adds two things the platform cannot compute: how well each fielder performs against left-handed versus right-handed batters, and how much of an outfielder's range comes from his reaction, his acceleration and the route he takes. Both would make the choice of which past play to copy more realistic.</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>The simulator can produce a 'dropped third strike' play in the situations where a real one is possible, at a rate consistent with real baseball data.</t>
+          <t>The fielder profile carries the batter-hand split and the outfield first-step measurements, and the fielding model uses them without breaking the accuracy checks.</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>No detailed implementation plan exists yet; the next step is to design how this fits into the existing pitch and catcher outcome logic.</t>
+          <t>Load Savant's outs above average and outfield jump files, add the columns to the fielder profile, tune the weights and re-run the checks. Needs the Savant loader first.</t>
         </is>
       </c>
     </row>
@@ -992,27 +992,27 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>SIM-532</t>
+          <t>SIM-533</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Add fielder split-by-batter-hand and first-step measurements</t>
+          <t>Add pitcher arm angle and spin-shape measurements</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>The simulator compares fielders using range and error rates it computes itself. Savant adds two things the platform cannot compute: how well each fielder performs against left-handed versus right-handed batters, and how much of an outfielder's range comes from his reaction, his acceleration and the route he takes. Both would make the choice of which past play to copy more realistic.</t>
+          <t>The simulator groups similar pitchers by the speed and movement of their pitches. Savant publishes the pitcher's arm angle in degrees, and how much of each pitch's spin actually moves the ball. Both describe the pitcher physically rather than by his results. This is the least certain of the Savant additions, because the pitcher model deliberately leaves out where the ball is released, and arm angle is closely related to that.</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>The fielder profile carries the batter-hand split and the outfield first-step measurements, and the fielding model uses them without breaking the accuracy checks.</t>
+          <t>A decision is recorded on whether arm angle belongs in the pitcher model, and any measurements that are adopted are stored, weighted and checked.</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Load Savant's outs above average and outfield jump files, add the columns to the fielder profile, tune the weights and re-run the checks. Needs the Savant loader first.</t>
+          <t>Review the release-point decision first. If arm angle is accepted, load Savant's arm angle, active spin and spin direction files, add them to the pitcher profile, then tune and re-check.</t>
         </is>
       </c>
     </row>
@@ -1024,27 +1024,27 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>SIM-533</t>
+          <t>SIM-478/479/480</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>Add pitcher arm angle and spin-shape measurements</t>
+          <t>Certify the outfield-fence / home-run boundary logic</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>The simulator groups similar pitchers by the speed and movement of their pitches. Savant publishes the pitcher's arm angle in degrees, and how much of each pitch's spin actually moves the ball. Both describe the pitcher physically rather than by his results. This is the least certain of the Savant additions, because the pitcher model deliberately leaves out where the ball is released, and arm angle is closely related to that.</t>
+          <t>When a batted ball heads toward the outfield wall, the simulator checks that specific ballpark's real fence distance and height to decide whether it is a home run or stays in play. The three pieces of this feature (a table of every park's fence measurements, a model of how far a ball actually flies, and the final wall-play check) have been built and wired in as part of a recent redesign, but they are still marked as pending their own dedicated accuracy test before being called fully certified.</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>A decision is recorded on whether arm angle belongs in the pitcher model, and any measurements that are adopted are stored, weighted and checked.</t>
+          <t>The fence-boundary logic passes a dedicated accuracy check on the platform's standard test set for home-run and wall-play outcomes.</t>
         </is>
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Review the release-point decision first. If arm angle is accepted, load Savant's arm angle, active spin and spin direction files, add them to the pitcher profile, then tune and re-check.</t>
+          <t>Run the standard accuracy test focused on home-run and wall-play outcomes, and close out any tuning it surfaces.</t>
         </is>
       </c>
     </row>
@@ -1056,27 +1056,27 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>SIM-478/479/480</t>
+          <t>SIM-451</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Certify the outfield-fence / home-run boundary logic</t>
+          <t>Re-check that every play-selection group has enough data</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>When a batted ball heads toward the outfield wall, the simulator checks that specific ballpark's real fence distance and height to decide whether it is a home run or stays in play. The three pieces of this feature (a table of every park's fence measurements, a model of how far a ball actually flies, and the final wall-play check) have been built and wired in as part of a recent redesign, but they are still marked as pending their own dedicated accuracy test before being called fully certified.</t>
+          <t>The simulator picks each pitch by first grouping similar past pitches into small buckets (based on things like the count and which bases have runners), then drawing an outcome from the most similar bucket. This check re-measures how many real pitches fall into each of the roughly 2,880 buckets, to make sure none is so small that its draw becomes unreliable. It needs to be re-run because the number of buckets is about to double once the new pitch-realism factors go live.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>The fence-boundary logic passes a dedicated accuracy check on the platform's standard test set for home-run and wall-play outcomes.</t>
+          <t>The bucket-size check has been re-run on the current data, and the platform has a documented minimum acceptable bucket size based on the results.</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>Run the standard accuracy test focused on home-run and wall-play outcomes, and close out any tuning it surfaces.</t>
+          <t>Re-run the existing bucket-coverage measurement script once the pitch-realism-factor rebuild finishes, and use its results to set the minimum bucket size.</t>
         </is>
       </c>
     </row>
@@ -1088,27 +1088,27 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>SIM-451</t>
+          <t>SIM-519</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Re-check that every play-selection group has enough data</t>
+          <t>Build the live, schedule-driven game day view</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>The simulator picks each pitch by first grouping similar past pitches into small buckets (based on things like the count and which bases have runners), then drawing an outcome from the most similar bucket. This check re-measures how many real pitches fall into each of the roughly 2,880 buckets, to make sure none is so small that its draw becomes unreliable. It needs to be re-run because the number of buckets is about to double once the new pitch-realism factors go live.</t>
+          <t>The public-facing screen that lists all of today's games should pull its list directly from Major League Baseball's own public schedule and mark each game as upcoming, in progress, or finished. Right now it pulls its game list only from the platform's own database, which can miss games or show stale information. This is a multi-part project; each part can be finished and checked off on its own.</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>The bucket-size check has been re-run on the current data, and the platform has a documented minimum acceptable bucket size based on the results.</t>
+          <t>The day view lists every game the league's real schedule shows for that day, with the correct status, sourced live from the league rather than only from the platform's own stored data.</t>
         </is>
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>Re-run the existing bucket-coverage measurement script once the pitch-realism-factor rebuild finishes, and use its results to set the minimum bucket size.</t>
+          <t>Build a connection to the league's public schedule feed, use it to drive the list of games shown, and keep layering the platform's simulations, projections, and odds on top of that live list.</t>
         </is>
       </c>
     </row>
@@ -1120,59 +1120,59 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>SIM-519</t>
+          <t>SIM-524</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Build the live, schedule-driven game day view</t>
+          <t>Fix the database lock that blocks nightly data rebuilds</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>The public-facing screen that lists all of today's games should pull its list directly from Major League Baseball's own public schedule and mark each game as upcoming, in progress, or finished. Right now it pulls its game list only from the platform's own database, which can miss games or show stale information. This is a multi-part project; each part can be finished and checked off on its own.</t>
+          <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>The day view lists every game the league's real schedule shows for that day, with the correct status, sourced live from the league rather than only from the platform's own stored data.</t>
+          <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
         </is>
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>Build a connection to the league's public schedule feed, use it to drive the list of games shown, and keep layering the platform's simulations, projections, and odds on top of that live list.</t>
+          <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="145" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>SIM-524</t>
+          <t>SIM-443d</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Fix the database lock that blocks nightly data rebuilds</t>
+          <t>Restrict what the SQL query tool can read</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>The main statistics database cannot be safely rewritten while the live application is running, because a background worker system quietly keeps a lock on the database file. The only current way to run a data rebuild is to shut down the whole live application first, which slows down every data-refresh task and adds operational risk.</t>
+          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>A data rebuild can run successfully while the live application keeps serving requests, with no manual shutdown step required.</t>
+          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
         </is>
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
-          <t>Change how the background worker system starts up so it no longer holds a lock on the database file that blocks rebuild scripts from writing to it.</t>
+          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
         </is>
       </c>
     </row>
@@ -1184,27 +1184,27 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>SIM-443d</t>
+          <t>SIM-443e</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Restrict what the SQL query tool can read</t>
+          <t>Turn on the read-only database connection for the SQL tool</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>The platform includes a tool that lets a user run their own read-only database queries from the website. It only blocks queries that would change data, but does not restrict which parts of the database can be read, so a user could query internal system tables that list other database accounts and their passwords.</t>
+          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>The SQL query tool only allows reading from the platform's approved data tables, and requests to read internal system tables are blocked.</t>
+          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
         </is>
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Add a list of allowed tables to the query tool's safety check, and reject any query that reaches outside that list.</t>
+          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
         </is>
       </c>
     </row>
@@ -1216,27 +1216,27 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>SIM-443e</t>
+          <t>SIM-443a</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Turn on the read-only database connection for the SQL tool</t>
+          <t>Stop exposing database ports to the network</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>The SQL query tool was built to use a separate, limited-permission database connection for safety, but the setting that turns that connection on is currently switched off, so the tool quietly falls back to the full administrator database connection instead.</t>
+          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>The SQL query tool is confirmed to be using the limited, read-only database connection rather than the administrator connection.</t>
+          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
         </is>
       </c>
       <c r="F22" s="19" t="inlineStr">
         <is>
-          <t>Turn on and set the read-only connection's configuration value, then confirm the tool uses it.</t>
+          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
         </is>
       </c>
     </row>
@@ -1248,27 +1248,27 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>SIM-443a</t>
+          <t>SIM-443b</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Stop exposing database ports to the network</t>
+          <t>Remove the default database password and admin access</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>The main database, the cache, and the application are all currently reachable from any computer on the network, not just the local machine, because their network connections are open to every network instead of limited to the local computer.</t>
+          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>The database, cache, and application ports are reachable only from the local machine, and the application still works normally.</t>
+          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
         </is>
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Change each service's network setting in the deployment configuration to bind only to the local machine's own address.</t>
+          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
         </is>
       </c>
     </row>
@@ -1280,27 +1280,27 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>SIM-443b</t>
+          <t>SIM-443c</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Remove the default database password and admin access</t>
+          <t>Require login on the API</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>The database's password is stored in plain, readable text in a file that is checked into the project's shared code, and the account using it has full administrator-level access rather than only the access it actually needs.</t>
+          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>The database password is no longer stored in the shared project files, and the application uses an account with only the specific permissions it needs.</t>
+          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
         </is>
       </c>
       <c r="F24" s="19" t="inlineStr">
         <is>
-          <t>Move the password into a secrets manager or environment variable outside the shared code, and create a limited-permission database account for the application.</t>
+          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
         </is>
       </c>
     </row>
@@ -1312,27 +1312,27 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>SIM-443c</t>
+          <t>SIM-443f</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Require login on the API</t>
+          <t>Secure the shared cache (Redis)</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>The programming interface (API) that the website and other tools use to pull data from the platform currently lets any request through with no login check whenever a certain setting is left unset, which is the default. This means anyone who can reach the server can pull the full pitch-by-pitch dataset with no credentials.</t>
+          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>Every route that provides data or triggers work requires a valid login by default, with no setting that silently disables that requirement.</t>
+          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
         </is>
       </c>
       <c r="F25" s="19" t="inlineStr">
         <is>
-          <t>Fix the login check so it fails closed (requires login) unless deliberately configured otherwise, and re-test that all data routes are covered.</t>
+          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
         </is>
       </c>
     </row>
@@ -1344,27 +1344,27 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>SIM-443f</t>
+          <t>SIM-525</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>Secure the shared cache (Redis)</t>
+          <t>Set up scheduled backups</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>The platform's shared, fast temporary-storage system (called Redis) is reachable from other computers on the local network with no password, and it stores cached data in a format that can run arbitrary code if it is tampered with. Together, this means someone who can reach the cache could plant tampered data that later runs on the server.</t>
+          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>The shared cache requires a password to connect, and it is no longer reachable from the network without one.</t>
+          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
         </is>
       </c>
       <c r="F26" s="19" t="inlineStr">
         <is>
-          <t>Set a password on the cache and restrict its network access the same way as the other services; consider switching away from a data format that can execute code.</t>
+          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
         </is>
       </c>
     </row>
@@ -1376,98 +1376,67 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>SIM-525</t>
+          <t>SIM-493</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>Set up scheduled backups</t>
+          <t>Break up the oversized simulation-loop code file</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>None of the platform's three data stores (the main statistics database, the game-simulation database, and the bundle of pre-computed data the simulator reads at startup) currently have any automatic backup. If any were lost or corrupted, rebuilding them from scratch would take roughly 12 hours of reprocessing.</t>
+          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (over 3,400 lines) as more features were added over time. This makes it harder to review and maintain safely. The team has deliberately postponed this cleanup until the in-progress pitch-speed and pitch-realism work settles down.</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>All three data stores back up automatically on a schedule, and a real restore from that backup has been tested successfully at least once.</t>
+          <t>The simulation-loop code is split into smaller, clearly-scoped files with no change in what the simulator actually does, confirmed by the platform's existing automated tests.</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>Set up a scheduled backup job for each data store and verify a real restore works before considering this finished.</t>
+          <t>Wait until the pitch-bucketing and pitch-realism-factor tickets are settled, then split the file into smaller modules by responsibility.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="115" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>SIM-493</t>
-        </is>
-      </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>Break up the oversized simulation-loop code file</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>The single code file that runs the pitch-by-pitch game simulation has grown very large (over 3,400 lines) as more features were added over time. This makes it harder to review and maintain safely. The team has deliberately postponed this cleanup until the in-progress pitch-speed and pitch-realism work settles down.</t>
-        </is>
-      </c>
-      <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>The simulation-loop code is split into smaller, clearly-scoped files with no change in what the simulator actually does, confirmed by the platform's existing automated tests.</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>Wait until the pitch-bucketing and pitch-realism-factor tickets are settled, then split the file into smaller modules by responsibility.</t>
-        </is>
-      </c>
+      <c r="A28" s="22" t="n"/>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
     </row>
     <row r="29" ht="100" customHeight="1">
-      <c r="A29" s="22" t="n"/>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
-      <c r="F29" s="22" t="n"/>
-    </row>
-    <row r="30" ht="100" customHeight="1">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Priority key:</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>P0 — drop everything</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
+      <c r="C29" s="25" t="inlineStr">
         <is>
           <t>P1 — next up</t>
         </is>
       </c>
-      <c r="D30" s="26" t="inlineStr">
+      <c r="D29" s="26" t="inlineStr">
         <is>
           <t>P2 — planned</t>
         </is>
       </c>
-      <c r="E30" s="27" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>P3 — later</t>
         </is>
       </c>
-      <c r="F30" s="28" t="n"/>
-    </row>
+      <c r="F29" s="28" t="n"/>
+    </row>
+    <row r="30" ht="100" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>